<commit_message>
feat: 初始化 2026-003-中AGV小车 项目
</commit_message>
<xml_diff>
--- a/Body/5-Office/BOM表.xlsx
+++ b/Body/5-Office/BOM表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\win-daolaj3j0nc\F\internal class\N2500-25N\N2571-YBJ\N2571-YBJ-2603\3-office文件\供应\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\win-daolaj3j0nc\F\internal class\N2500-25N\N2571-YBJ\N2571-YBJ-2604\3-office文件\供应\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E153A097-F61A-4577-ACB2-D0A134EE198D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9262237-BA8F-4BBB-96AB-C003ABA7DB8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="149">
   <si>
     <r>
       <rPr>
@@ -485,10 +485,6 @@
     </r>
   </si>
   <si>
-    <t>Optimized
-优选等级</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -632,9 +628,6 @@
     <t>1225-左梁</t>
   </si>
   <si>
-    <t>1215-平头圆柱销</t>
-  </si>
-  <si>
     <t>1212-销</t>
   </si>
   <si>
@@ -693,9 +686,6 @@
   </si>
   <si>
     <t>0116-内六角平圆头螺钉-GBT70.2-2015_M5X12</t>
-  </si>
-  <si>
-    <t>0124-钢轧带</t>
   </si>
   <si>
     <t>0125-电器架</t>
@@ -798,39 +788,6 @@
   </si>
   <si>
     <r>
-      <t>【淘宝】</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>7</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>天无理由退货</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> https://e.tb.cn/h.7mlCpa3CT8fUR1f?tk=w2zsUfW92Ot </t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>【淘宝】大促价保</t>
     </r>
     <r>
@@ -848,16 +805,471 @@
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
   <si>
-    <t>直径10</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
     <t>M10</t>
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t>3.82</t>
+    <t>2111-电箱din导轨 130</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>【淘宝】假一赔四</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> https://e.tb.cn/h.7MJcgNyqDq0lb4x?tk=nxhCUgh63I7 CZ193 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>304</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>不锈钢垫片圆形加大加厚金属螺丝平垫圈超薄介子华司平垫大全」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>点击链接直接打开</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>或者</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>淘宝搜索直接打开</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>【淘宝】退货运费险</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> https://e.tb.cn/h.7Lm8guSC0Ux0SfB?tk=6AuNUghRivr CZ028 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>「进口模具弹簧高强度耐高温矩形扁线压缩磨具压簧黄蓝红绿棕褐茶色」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>点击链接直接打开</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>或者</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>淘宝搜索直接打开</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>【淘宝】大促价保</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> https://e.tb.cn/h.7MJ4SWmHd5yGuXb?tk=qO5IUghjzTA CZ028 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>「</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>寸重型万向轮</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>低重心尼龙脚轮</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>寸双轮轱辘</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>寸推车带刹加重轮子」</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>点击链接直接打开</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>或者</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>淘宝搜索直接打开</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0126-miniPC电源</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>19V10A</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?id=553788314091&amp;last_time=1768143784&amp;mi_id=0000i7eOrBKgQD4GnhXhm9jjujyg938wVli_lWGICSqSW3s&amp;scm=1007.13982.82927.0&amp;skuId=4092429570913&amp;spm=tbpc.mytb_footmark.item.goods&amp;upStreamPrice=3915</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0127-变压器</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>24V6.35A</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>24V15A</t>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1563820041%3AH%3AjEXVXFz29uWhSPA32SdLxq18tbGVRP6N%3Ab1e44a53e68312397166bdb38376f31f&amp;ali_trackid=318_b1e44a53e68312397166bdb38376f31f&amp;id=668804973431&amp;mi_id=0000kh4JsEhs_IKQwaZwLe5GPzZBrKEtnqIAl4nMzgEcpGs&amp;mm_sceneid=0_0_2198670068_0&amp;priceTId=213e097817677727727551092e11ab&amp;skuId=6072168990782&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%220ce0092ebee4bb5c990e1ed0aae83472%22%7D&amp;xxc=ad_ztc</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0128-屏幕电源</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0129-接触器</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>12A, 24 V</t>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?abbucket=15&amp;id=684180101591&amp;mi_id=0000kHsnKO9vrl_xXRKAYuWwfk1ZxpJzkY1oGgmAntBdN2A&amp;ns=1&amp;priceTId=215040db17693197452846906e10bd&amp;skuId=5066190559427&amp;spm=a21n57.1.hoverItem.13&amp;utparam=%7B%22aplus_abtest%22%3A%2200fb48171d68baf920a6c2997ba800f5%22%7D&amp;xxc=taobaoSearch</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0130-空开</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?abbucket=15&amp;id=885444239746&amp;mi_id=00004gN7JSgLTLqH9NscZa5BV-fDjGIRhn7dS2llqgBEm-I&amp;ns=1&amp;priceTId=215040db17693199893824488e10bd&amp;skuId=5729109569961&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%220d184a79d8dee207c56cd615483888e0%22%7D&amp;xxc=taobaoSearch</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.jndz021.com/dc/132（淘宝没有货源，在官网上采购）</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1202830031%3AH%3A5NEVSZWkfH5vk10Gx8WsEg%3D%3D%3A0e3224a199436b146fadd1013df40d50&amp;ali_trackid=282_0e3224a199436b146fadd1013df40d50&amp;id=589213401941&amp;mi_id=0000tXboOyQ6vKwx8WiuBo_0I904yCwGgBZQ-DEtp9Eidvc&amp;mm_sceneid=1_0_343370108_0&amp;priceTId=214782f517694062736734983e1fe1&amp;skuId=4715656587781&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%2243f96ce6df79319aabdbd4973057b1b5%22%7D&amp;xxc=ad_ztc</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0132-焊枪（一套）</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0133-电池</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>电池客服：13662632158</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>48V20AH</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0134-仙工控制器</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>已经购买</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0135-激光雷达</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0135-导航雷达</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>0131-接线端子</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>PT2.5-QUATTRO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>灰色</t>
+    </r>
+  </si>
+  <si>
+    <t>https://item.taobao.com/item.htm?ali_refid=a3_430673_1006%3A1109974134%3AH%3AS9mt8%2FS9IPRAnlGXK23dCRerfi2%2BAYZj%3A75421c7a1bf937df626379b8de81db84&amp;ali_trackid=282_75421c7a1bf937df626379b8de81db84&amp;id=774427618182&amp;loginBonus=1&amp;mi_id=0000OtzXamOT9vAra9TbUQiBvRLBsdZJRcmzsekmz3yUyS0&amp;mm_sceneid=1_0_99588015_0&amp;priceTId=2150467817696032421462002e22b0&amp;skuId=5300832301565&amp;spm=a21n57.sem.item.4&amp;utparam=%7B%22aplus_abtest%22%3A%22c7bbb9e8de08729fc098be83e797fb13%22%7D&amp;xxc=ad_ztc</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>1312-电机</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>是否验收</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>对</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>3129-顶板</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>269</t>
     </r>
     <r>
       <rPr>
@@ -872,7 +1284,7 @@
   </si>
   <si>
     <r>
-      <t>1.8</t>
+      <t>118</t>
     </r>
     <r>
       <rPr>
@@ -886,15 +1298,9 @@
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
   <si>
-    <t>2111-电箱din导轨 130</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>【淘宝】7天无理由退货 https://e.tb.cn/h.7LmgfPhmD1WJjfq?tk=UthlUghUNJc CZ321 「国标卡固氧化C45导轨U型TH35MM宽断路器端子空开电气加厚铝卡轨条」
-点击链接直接打开 或者 淘宝搜索直接打开</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
+    <r>
+      <t>231</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -902,15 +1308,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>【淘宝】假一赔四</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> https://e.tb.cn/h.7MJcgNyqDq0lb4x?tk=nxhCUgh63I7 CZ193 </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>160</t>
     </r>
     <r>
       <rPr>
@@ -919,15 +1323,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>「</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>304</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>83</t>
     </r>
     <r>
       <rPr>
@@ -936,16 +1338,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>不锈钢垫片圆形加大加厚金属螺丝平垫圈超薄介子华司平垫大全」</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>63.5</t>
     </r>
     <r>
       <rPr>
@@ -954,15 +1353,46 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>点击链接直接打开</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>还未咨询</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>钣金统一计价</t>
+  </si>
+  <si>
+    <t>钣金统一计价</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>已经购买</t>
+  </si>
+  <si>
+    <r>
+      <t>【淘宝】大促价保</t>
     </r>
     <r>
       <rPr>
+        <b/>
         <sz val="11"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve"> https://e.tb.cn/h.7mOc2Ra9KZEBda1?tk=7f3aUfWpWek</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>钣金件合计</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>20.2</t>
     </r>
     <r>
       <rPr>
@@ -971,15 +1401,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>或者</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>40.4</t>
     </r>
     <r>
       <rPr>
@@ -988,11 +1416,30 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>淘宝搜索直接打开</t>
+      <t>元</t>
     </r>
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
   <si>
+    <t>加工件统一计价</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>加工件合计</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>1215-平头圆柱销</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>直径10x45</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>5</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -1000,15 +1447,25 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>【淘宝】退货运费险</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> https://e.tb.cn/h.7Lm8guSC0Ux0SfB?tk=6AuNUghRivr CZ028 </t>
+      <t>个</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>组</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>7.05元</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>细则</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>7.05</t>
     </r>
     <r>
       <rPr>
@@ -1017,16 +1474,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>「进口模具弹簧高强度耐高温矩形扁线压缩磨具压簧黄蓝红绿棕褐茶色」</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>4.37</t>
     </r>
     <r>
       <rPr>
@@ -1035,15 +1489,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>点击链接直接打开</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>4.64</t>
     </r>
     <r>
       <rPr>
@@ -1052,15 +1504,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>或者</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>13.92</t>
     </r>
     <r>
       <rPr>
@@ -1069,11 +1519,22 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>淘宝搜索直接打开</t>
+      <t>元</t>
     </r>
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
   <si>
+    <t>https://item.taobao.com/item.htm?abbucket=11&amp;id=749064062909&amp;mi_id=0000D_lgnxXXWYg6uIU45wamE0Zv9ob04zflYhEBkPv_GQo&amp;ns=1&amp;skuId=5394057435750&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%220457ff662cd3c9532cc0680e1a87dd2b%22%7D&amp;xxc=taobaoSearch</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>10*30*2</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.13</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -1081,15 +1542,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>【淘宝】大促价保</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> https://e.tb.cn/h.7MJ4SWmHd5yGuXb?tk=qO5IUghjzTA CZ028 </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1.58</t>
     </r>
     <r>
       <rPr>
@@ -1098,15 +1557,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>「</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>1</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>2.73</t>
     </r>
     <r>
       <rPr>
@@ -1115,15 +1572,13 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>寸重型万向轮</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>5.46</t>
     </r>
     <r>
       <rPr>
@@ -1132,217 +1587,34 @@
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>低重心尼龙脚轮</t>
+      <t>元</t>
+    </r>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>个</t>
+  </si>
+  <si>
+    <t>个</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <t>【淘宝】https://e.tb.cn/h.iJUYQFq3IH6uaaV?tk=fsBd5SyIRlW</t>
+    <phoneticPr fontId="61" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">    360</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
+        <sz val="12"/>
         <rFont val="宋体"/>
         <family val="2"/>
         <charset val="134"/>
       </rPr>
-      <t>寸双轮轱辘</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> 3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>寸推车带刹加重轮子」</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>点击链接直接打开</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>或者</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>淘宝搜索直接打开</t>
-    </r>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0126-miniPC电源</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>19V10A</t>
-  </si>
-  <si>
-    <t>https://item.taobao.com/item.htm?id=553788314091&amp;last_time=1768143784&amp;mi_id=0000i7eOrBKgQD4GnhXhm9jjujyg938wVli_lWGICSqSW3s&amp;scm=1007.13982.82927.0&amp;skuId=4092429570913&amp;spm=tbpc.mytb_footmark.item.goods&amp;upStreamPrice=3915</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0127-变压器</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>24V6.35A</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>24V15A</t>
-  </si>
-  <si>
-    <t>https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1563820041%3AH%3AjEXVXFz29uWhSPA32SdLxq18tbGVRP6N%3Ab1e44a53e68312397166bdb38376f31f&amp;ali_trackid=318_b1e44a53e68312397166bdb38376f31f&amp;id=668804973431&amp;mi_id=0000kh4JsEhs_IKQwaZwLe5GPzZBrKEtnqIAl4nMzgEcpGs&amp;mm_sceneid=0_0_2198670068_0&amp;priceTId=213e097817677727727551092e11ab&amp;skuId=6072168990782&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%220ce0092ebee4bb5c990e1ed0aae83472%22%7D&amp;xxc=ad_ztc</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0128-屏幕电源</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0129-接触器</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>12A, 24 V</t>
-  </si>
-  <si>
-    <t>https://item.taobao.com/item.htm?abbucket=15&amp;id=684180101591&amp;mi_id=0000kHsnKO9vrl_xXRKAYuWwfk1ZxpJzkY1oGgmAntBdN2A&amp;ns=1&amp;priceTId=215040db17693197452846906e10bd&amp;skuId=5066190559427&amp;spm=a21n57.1.hoverItem.13&amp;utparam=%7B%22aplus_abtest%22%3A%2200fb48171d68baf920a6c2997ba800f5%22%7D&amp;xxc=taobaoSearch</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0130-空开</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://item.taobao.com/item.htm?abbucket=15&amp;id=885444239746&amp;mi_id=00004gN7JSgLTLqH9NscZa5BV-fDjGIRhn7dS2llqgBEm-I&amp;ns=1&amp;priceTId=215040db17693199893824488e10bd&amp;skuId=5729109569961&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%220d184a79d8dee207c56cd615483888e0%22%7D&amp;xxc=taobaoSearch</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://www.jndz021.com/dc/132（淘宝没有货源，在官网上采购）</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1202830031%3AH%3A5NEVSZWkfH5vk10Gx8WsEg%3D%3D%3A0e3224a199436b146fadd1013df40d50&amp;ali_trackid=282_0e3224a199436b146fadd1013df40d50&amp;id=589213401941&amp;mi_id=0000tXboOyQ6vKwx8WiuBo_0I904yCwGgBZQ-DEtp9Eidvc&amp;mm_sceneid=1_0_343370108_0&amp;priceTId=214782f517694062736734983e1fe1&amp;skuId=4715656587781&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%2243f96ce6df79319aabdbd4973057b1b5%22%7D&amp;xxc=ad_ztc</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0132-焊枪（一套）</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0133-电池</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>电池客服：13662632158</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>48V20AH</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0134-仙工控制器</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>已经购买</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0135-激光雷达</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0135-导航雷达</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>0131-接线端子</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>PT2.5-QUATTRO</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="宋体"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>灰色</t>
-    </r>
-  </si>
-  <si>
-    <t>https://item.taobao.com/item.htm?ali_refid=a3_430673_1006%3A1109974134%3AH%3AS9mt8%2FS9IPRAnlGXK23dCRerfi2%2BAYZj%3A75421c7a1bf937df626379b8de81db84&amp;ali_trackid=282_75421c7a1bf937df626379b8de81db84&amp;id=774427618182&amp;loginBonus=1&amp;mi_id=0000OtzXamOT9vAra9TbUQiBvRLBsdZJRcmzsekmz3yUyS0&amp;mm_sceneid=1_0_99588015_0&amp;priceTId=2150467817696032421462002e22b0&amp;skuId=5300832301565&amp;spm=a21n57.sem.item.4&amp;utparam=%7B%22aplus_abtest%22%3A%22c7bbb9e8de08729fc098be83e797fb13%22%7D&amp;xxc=ad_ztc</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>1312-电机</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>是否验收</t>
-    <phoneticPr fontId="61" type="noConversion"/>
-  </si>
-  <si>
-    <t>对</t>
+      <t>元</t>
+    </r>
     <phoneticPr fontId="61" type="noConversion"/>
   </si>
 </sst>
@@ -1362,7 +1634,7 @@
     <numFmt numFmtId="182" formatCode="0.00_ "/>
     <numFmt numFmtId="183" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="69" x14ac:knownFonts="1">
+  <fonts count="72" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1818,6 +2090,27 @@
     <font>
       <sz val="11"/>
       <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="宋体"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
@@ -3001,7 +3294,7 @@
     </xf>
     <xf numFmtId="176" fontId="67" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="83">
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3149,9 +3442,87 @@
     <xf numFmtId="181" fontId="65" fillId="33" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="65" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="64" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="69" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="70" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="65" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="67" fillId="4" borderId="1" xfId="266" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="70" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="62" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="62" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="62" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3165,63 +3536,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="62" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="62" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="62" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3879,7 +4193,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:WVF1221"/>
+  <dimension ref="A1:WVF1220"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="5.625" style="5" customWidth="1"/>
@@ -5224,174 +5538,174 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="51"/>
+      <c r="A1" s="61"/>
       <c r="B1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="53" t="s">
+      <c r="C1" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="53"/>
+      <c r="D1" s="79"/>
       <c r="E1" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="59"/>
-      <c r="G1" s="51" t="s">
+      <c r="F1" s="60"/>
+      <c r="G1" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="51"/>
+      <c r="H1" s="61"/>
       <c r="I1" s="11"/>
       <c r="J1" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="59"/>
-      <c r="L1" s="51" t="s">
+      <c r="K1" s="60"/>
+      <c r="L1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="51"/>
+      <c r="M1" s="61"/>
       <c r="N1" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="71"/>
-      <c r="P1" s="59"/>
+      <c r="O1" s="59"/>
+      <c r="P1" s="60"/>
     </row>
     <row r="2" spans="1:16" s="1" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="51"/>
+      <c r="A2" s="61"/>
       <c r="B2" s="12"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="62" t="s">
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="G2" s="65">
+      <c r="F2" s="70"/>
+      <c r="G2" s="73">
         <v>1</v>
       </c>
-      <c r="H2" s="65"/>
-      <c r="I2" s="66"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="74"/>
       <c r="J2" s="58"/>
-      <c r="K2" s="59"/>
+      <c r="K2" s="60"/>
       <c r="L2" s="58"/>
-      <c r="M2" s="59"/>
+      <c r="M2" s="60"/>
       <c r="N2" s="58"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="60"/>
     </row>
     <row r="3" spans="1:16" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="51"/>
+      <c r="A3" s="61"/>
       <c r="B3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="66"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="79"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="74"/>
       <c r="J3" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="K3" s="59"/>
-      <c r="L3" s="51" t="s">
+      <c r="K3" s="60"/>
+      <c r="L3" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="51"/>
+      <c r="M3" s="61"/>
       <c r="N3" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="71"/>
-      <c r="P3" s="59"/>
+      <c r="O3" s="59"/>
+      <c r="P3" s="60"/>
     </row>
     <row r="4" spans="1:16" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="52"/>
+      <c r="A4" s="78"/>
       <c r="B4" s="12"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="52" t="s">
+      <c r="C4" s="81"/>
+      <c r="D4" s="81"/>
+      <c r="E4" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="52"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="57"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="70"/>
       <c r="J4" s="58"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="52"/>
-      <c r="M4" s="52"/>
+      <c r="K4" s="60"/>
+      <c r="L4" s="78"/>
+      <c r="M4" s="78"/>
       <c r="N4" s="58"/>
-      <c r="O4" s="71"/>
-      <c r="P4" s="59"/>
+      <c r="O4" s="59"/>
+      <c r="P4" s="60"/>
     </row>
     <row r="5" spans="1:16" s="2" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="72" t="s">
+      <c r="A5" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="73" t="s">
+      <c r="B5" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="74" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="68" t="s">
+      <c r="C5" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="68" t="s">
+      <c r="E5" s="66" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="51" t="s">
+      <c r="F5" s="61" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="51"/>
-      <c r="H5" s="67" t="s">
-        <v>74</v>
-      </c>
-      <c r="I5" s="51" t="s">
+      <c r="G5" s="61"/>
+      <c r="H5" s="75" t="s">
+        <v>71</v>
+      </c>
+      <c r="I5" s="61" t="s">
         <v>20</v>
       </c>
-      <c r="J5" s="51" t="s">
+      <c r="J5" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="69" t="s">
-        <v>118</v>
-      </c>
-      <c r="L5" s="51" t="s">
+      <c r="K5" s="76" t="s">
+        <v>110</v>
+      </c>
+      <c r="L5" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="51" t="s">
+      <c r="M5" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="N5" s="60" t="s">
+      <c r="N5" s="67" t="s">
+        <v>134</v>
+      </c>
+      <c r="O5" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="O5" s="51" t="s">
+      <c r="P5" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="P5" s="51" t="s">
+    </row>
+    <row r="6" spans="1:16" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.15">
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="11" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" s="2" customFormat="1" ht="30" x14ac:dyDescent="0.15">
-      <c r="A6" s="72"/>
-      <c r="B6" s="73"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="11" t="s">
+      <c r="G6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H6" s="68"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
-      <c r="K6" s="70"/>
-      <c r="L6" s="51"/>
-      <c r="M6" s="51"/>
-      <c r="N6" s="61"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
+      <c r="H6" s="66"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="77"/>
+      <c r="L6" s="61"/>
+      <c r="M6" s="61"/>
+      <c r="N6" s="68"/>
+      <c r="O6" s="61"/>
+      <c r="P6" s="61"/>
     </row>
     <row r="7" spans="1:16" s="3" customFormat="1" ht="78.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="14">
@@ -5402,26 +5716,30 @@
         <v>1121</v>
       </c>
       <c r="D7" s="35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E7" s="18"/>
       <c r="F7" s="15"/>
       <c r="G7" s="15"/>
       <c r="H7" s="38" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I7" s="15">
         <v>1</v>
       </c>
-      <c r="J7" s="15"/>
+      <c r="J7" s="57" t="s">
+        <v>146</v>
+      </c>
       <c r="K7" s="17"/>
       <c r="L7" s="42" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="M7" s="16"/>
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
+      <c r="P7" s="54" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="8" spans="1:16" s="4" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="14">
@@ -5432,26 +5750,30 @@
         <v>2122</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8" s="22"/>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
       <c r="H8" s="38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I8" s="20">
         <v>4</v>
       </c>
-      <c r="J8" s="20"/>
+      <c r="J8" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K8" s="21"/>
       <c r="L8" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
+      <c r="P8" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="9" spans="1:16" s="4" customFormat="1" ht="99" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="14">
@@ -5462,10 +5784,10 @@
         <v>1113</v>
       </c>
       <c r="D9" s="35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
@@ -5473,17 +5795,21 @@
       <c r="I9" s="20">
         <v>34</v>
       </c>
-      <c r="J9" s="20"/>
+      <c r="J9" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K9" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L9" s="50" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M9" s="27"/>
       <c r="N9" s="27"/>
       <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
+      <c r="P9" s="51" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="10" spans="1:16" s="4" customFormat="1" ht="139.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="14">
@@ -5494,10 +5820,10 @@
         <v>1312</v>
       </c>
       <c r="D10" s="35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F10" s="27"/>
       <c r="G10" s="20"/>
@@ -5505,17 +5831,21 @@
       <c r="I10" s="24">
         <v>14</v>
       </c>
-      <c r="J10" s="20"/>
+      <c r="J10" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K10" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L10" s="50" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M10" s="27"/>
       <c r="N10" s="27"/>
       <c r="O10" s="27"/>
-      <c r="P10" s="27"/>
+      <c r="P10" s="51" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="11" spans="1:16" s="4" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="14">
@@ -5526,26 +5856,30 @@
         <v>1221</v>
       </c>
       <c r="D11" s="35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11" s="22"/>
       <c r="F11" s="27"/>
       <c r="G11" s="20"/>
       <c r="H11" s="37" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I11" s="24">
         <v>2</v>
       </c>
-      <c r="J11" s="20"/>
+      <c r="J11" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K11" s="21"/>
       <c r="L11" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M11" s="27"/>
       <c r="N11" s="27"/>
       <c r="O11" s="27"/>
-      <c r="P11" s="27"/>
+      <c r="P11" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="12" spans="1:16" s="4" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="14">
@@ -5556,26 +5890,30 @@
         <v>1222</v>
       </c>
       <c r="D12" s="35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" s="22"/>
       <c r="F12" s="27"/>
       <c r="G12" s="20"/>
       <c r="H12" s="37" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I12" s="24">
         <v>2</v>
       </c>
-      <c r="J12" s="20"/>
+      <c r="J12" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K12" s="21"/>
       <c r="L12" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M12" s="27"/>
       <c r="N12" s="27"/>
       <c r="O12" s="27"/>
-      <c r="P12" s="27"/>
+      <c r="P12" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="13" spans="1:16" s="4" customFormat="1" ht="127.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="14">
@@ -5586,24 +5924,34 @@
         <v>1213</v>
       </c>
       <c r="D13" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="22"/>
+        <v>34</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>140</v>
+      </c>
       <c r="F13" s="27"/>
       <c r="G13" s="20"/>
       <c r="H13" s="22"/>
       <c r="I13" s="24">
-        <v>4</v>
-      </c>
-      <c r="J13" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J13" s="55" t="s">
+        <v>132</v>
+      </c>
       <c r="K13" s="21"/>
       <c r="L13" s="44" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="M13" s="27"/>
-      <c r="N13" s="27"/>
-      <c r="O13" s="27"/>
-      <c r="P13" s="27"/>
+      <c r="N13" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="O13" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="P13" s="27" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="14" spans="1:16" s="4" customFormat="1" ht="87.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="14">
@@ -5614,13 +5962,13 @@
         <v>1224</v>
       </c>
       <c r="D14" s="35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E14" s="22"/>
       <c r="F14" s="15"/>
       <c r="G14" s="20"/>
       <c r="H14" s="39" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I14" s="40">
         <v>2</v>
@@ -5628,12 +5976,14 @@
       <c r="J14" s="15"/>
       <c r="K14" s="28"/>
       <c r="L14" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M14" s="27"/>
       <c r="N14" s="27"/>
       <c r="O14" s="27"/>
-      <c r="P14" s="27"/>
+      <c r="P14" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="15" spans="1:16" s="4" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="14">
@@ -5644,24 +5994,32 @@
         <v>1214</v>
       </c>
       <c r="D15" s="35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E15" s="22"/>
       <c r="F15" s="27"/>
       <c r="G15" s="20"/>
       <c r="H15" s="22"/>
       <c r="I15" s="24">
-        <v>4</v>
-      </c>
-      <c r="J15" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J15" s="55" t="s">
+        <v>132</v>
+      </c>
       <c r="K15" s="21"/>
       <c r="L15" s="44" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-      <c r="O15" s="27"/>
-      <c r="P15" s="27"/>
+      <c r="N15" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="O15" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="P15" s="27" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="16" spans="1:16" s="4" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="14">
@@ -5672,7 +6030,7 @@
         <v>1218</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E16" s="22"/>
       <c r="F16" s="27"/>
@@ -5681,15 +6039,21 @@
       <c r="I16" s="24">
         <v>2</v>
       </c>
-      <c r="J16" s="20"/>
+      <c r="J16" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K16" s="21"/>
       <c r="L16" s="44" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="M16" s="27"/>
       <c r="N16" s="27"/>
-      <c r="O16" s="27"/>
-      <c r="P16" s="27"/>
+      <c r="O16" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="P16" s="27" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="17" spans="1:16" s="4" customFormat="1" ht="52.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="14">
@@ -5700,26 +6064,30 @@
         <v>1225</v>
       </c>
       <c r="D17" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E17" s="22"/>
       <c r="F17" s="27"/>
       <c r="G17" s="20"/>
       <c r="H17" s="48" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I17" s="24">
         <v>1</v>
       </c>
-      <c r="J17" s="20"/>
+      <c r="J17" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K17" s="21"/>
       <c r="L17" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M17" s="27"/>
       <c r="N17" s="27"/>
       <c r="O17" s="27"/>
-      <c r="P17" s="27"/>
+      <c r="P17" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="18" spans="1:16" s="4" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="14">
@@ -5729,27 +6097,35 @@
       <c r="C18" s="20">
         <v>1215</v>
       </c>
-      <c r="D18" s="35" t="s">
-        <v>40</v>
+      <c r="D18" s="36" t="s">
+        <v>129</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>82</v>
+        <v>130</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
       <c r="H18" s="22"/>
       <c r="I18" s="20">
-        <v>2</v>
-      </c>
-      <c r="J18" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J18" s="55" t="s">
+        <v>132</v>
+      </c>
       <c r="K18" s="21"/>
       <c r="L18" s="43" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
+      <c r="N18" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="O18" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="P18" s="27" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="19" spans="1:16" ht="51.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="14">
@@ -5760,26 +6136,34 @@
         <v>1212</v>
       </c>
       <c r="D19" s="35" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
       <c r="H19" s="22"/>
       <c r="I19" s="20">
-        <v>2</v>
-      </c>
-      <c r="J19" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J19" s="55" t="s">
+        <v>132</v>
+      </c>
       <c r="K19" s="21"/>
       <c r="L19" s="43" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="M19" s="27"/>
-      <c r="N19" s="27"/>
-      <c r="O19" s="27"/>
-      <c r="P19" s="27"/>
+      <c r="N19" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="O19" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="P19" s="27" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="20" spans="1:16" ht="109.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="14">
@@ -5790,10 +6174,10 @@
         <v>1217</v>
       </c>
       <c r="D20" s="35" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
@@ -5801,18 +6185,20 @@
       <c r="I20" s="20">
         <v>8</v>
       </c>
-      <c r="J20" s="20"/>
+      <c r="J20" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K20" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L20" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M20" s="27"/>
       <c r="N20" s="27"/>
       <c r="O20" s="27"/>
-      <c r="P20" s="27" t="s">
-        <v>84</v>
+      <c r="P20" s="51" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="120.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -5824,10 +6210,10 @@
         <v>1218</v>
       </c>
       <c r="D21" s="35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
@@ -5835,18 +6221,20 @@
       <c r="I21" s="20">
         <v>8</v>
       </c>
-      <c r="J21" s="20"/>
+      <c r="J21" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K21" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L21" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M21" s="27"/>
       <c r="N21" s="27"/>
       <c r="O21" s="27"/>
-      <c r="P21" s="27" t="s">
-        <v>85</v>
+      <c r="P21" s="51" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="111" customHeight="1" x14ac:dyDescent="0.15">
@@ -5858,10 +6246,10 @@
         <v>1216</v>
       </c>
       <c r="D22" s="35" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
@@ -5869,17 +6257,21 @@
       <c r="I22" s="20">
         <v>2</v>
       </c>
-      <c r="J22" s="20"/>
+      <c r="J22" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K22" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L22" s="50" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M22" s="27"/>
       <c r="N22" s="27"/>
       <c r="O22" s="27"/>
-      <c r="P22" s="27"/>
+      <c r="P22" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="23" spans="1:16" ht="58.5" x14ac:dyDescent="0.15">
       <c r="A23" s="14">
@@ -5890,7 +6282,7 @@
         <v>1223</v>
       </c>
       <c r="D23" s="35" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="20"/>
@@ -5899,15 +6291,19 @@
       <c r="I23" s="20">
         <v>1</v>
       </c>
-      <c r="J23" s="20"/>
+      <c r="J23" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K23" s="21"/>
       <c r="L23" s="42" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="M23" s="27"/>
       <c r="N23" s="27"/>
       <c r="O23" s="27"/>
-      <c r="P23" s="27"/>
+      <c r="P23" s="51" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="14">
@@ -5918,7 +6314,7 @@
         <v>1521</v>
       </c>
       <c r="D24" s="35" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E24" s="22"/>
       <c r="F24" s="20"/>
@@ -5927,17 +6323,21 @@
       <c r="I24" s="20">
         <v>1</v>
       </c>
-      <c r="J24" s="20"/>
+      <c r="J24" s="46" t="s">
+        <v>145</v>
+      </c>
       <c r="K24" s="21"/>
       <c r="L24" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M24" s="27">
         <v>1</v>
       </c>
       <c r="N24" s="27"/>
       <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
+      <c r="P24" s="51" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="25" spans="1:16" ht="117" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="14">
@@ -5948,10 +6348,10 @@
         <v>1515</v>
       </c>
       <c r="D25" s="35" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F25" s="20"/>
       <c r="G25" s="20"/>
@@ -5959,17 +6359,21 @@
       <c r="I25" s="20">
         <v>6</v>
       </c>
-      <c r="J25" s="20"/>
+      <c r="J25" s="46" t="s">
+        <v>145</v>
+      </c>
       <c r="K25" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L25" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M25" s="27"/>
       <c r="N25" s="27"/>
       <c r="O25" s="27"/>
-      <c r="P25" s="27"/>
+      <c r="P25" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="26" spans="1:16" ht="122.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="14">
@@ -5980,10 +6384,10 @@
         <v>1516</v>
       </c>
       <c r="D26" s="35" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="20"/>
@@ -5991,17 +6395,21 @@
       <c r="I26" s="20">
         <v>2</v>
       </c>
-      <c r="J26" s="20"/>
+      <c r="J26" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K26" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L26" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M26" s="27"/>
       <c r="N26" s="27"/>
       <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
+      <c r="P26" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="27" spans="1:16" ht="96" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="14">
@@ -6012,7 +6420,7 @@
         <v>1522</v>
       </c>
       <c r="D27" s="35" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E27" s="22"/>
       <c r="F27" s="20"/>
@@ -6021,17 +6429,21 @@
       <c r="I27" s="20">
         <v>1</v>
       </c>
-      <c r="J27" s="20"/>
+      <c r="J27" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K27" s="21"/>
       <c r="L27" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M27" s="27">
         <v>1</v>
       </c>
       <c r="N27" s="27"/>
       <c r="O27" s="27"/>
-      <c r="P27" s="27"/>
+      <c r="P27" s="51" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="28" spans="1:16" ht="129.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="14">
@@ -6042,10 +6454,10 @@
         <v>1577</v>
       </c>
       <c r="D28" s="35" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F28" s="20"/>
       <c r="G28" s="20"/>
@@ -6053,17 +6465,21 @@
       <c r="I28" s="20">
         <v>18</v>
       </c>
-      <c r="J28" s="20"/>
+      <c r="J28" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K28" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L28" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M28" s="27"/>
       <c r="N28" s="27"/>
       <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
+      <c r="P28" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="29" spans="1:16" ht="129" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="14">
@@ -6074,7 +6490,7 @@
         <v>1411</v>
       </c>
       <c r="D29" s="35" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E29" s="22"/>
       <c r="F29" s="20"/>
@@ -6083,17 +6499,23 @@
       <c r="I29" s="20">
         <v>2</v>
       </c>
-      <c r="J29" s="20"/>
+      <c r="J29" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K29" s="21"/>
       <c r="L29" s="44" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="M29" s="27"/>
       <c r="N29" s="27"/>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-    </row>
-    <row r="30" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="O29" s="27" t="s">
+        <v>125</v>
+      </c>
+      <c r="P29" s="27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A30" s="14">
         <v>24</v>
       </c>
@@ -6102,7 +6524,7 @@
         <v>1421</v>
       </c>
       <c r="D30" s="35" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E30" s="22"/>
       <c r="F30" s="20"/>
@@ -6111,19 +6533,23 @@
       <c r="I30" s="20">
         <v>2</v>
       </c>
-      <c r="J30" s="20"/>
+      <c r="J30" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K30" s="21"/>
       <c r="L30" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M30" s="27">
         <v>1</v>
       </c>
       <c r="N30" s="27"/>
       <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-    </row>
-    <row r="31" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P30" s="51" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A31" s="14">
         <v>25</v>
       </c>
@@ -6132,7 +6558,7 @@
         <v>1621</v>
       </c>
       <c r="D31" s="35" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E31" s="22"/>
       <c r="F31" s="20"/>
@@ -6141,15 +6567,19 @@
       <c r="I31" s="20">
         <v>1</v>
       </c>
-      <c r="J31" s="20"/>
+      <c r="J31" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K31" s="21"/>
       <c r="L31" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M31" s="27"/>
       <c r="N31" s="27"/>
       <c r="O31" s="27"/>
-      <c r="P31" s="27"/>
+      <c r="P31" s="51" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="32" spans="1:16" ht="114.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="14">
@@ -6160,10 +6590,10 @@
         <v>1713</v>
       </c>
       <c r="D32" s="35" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F32" s="20"/>
       <c r="G32" s="20"/>
@@ -6171,17 +6601,21 @@
       <c r="I32" s="20">
         <v>8</v>
       </c>
-      <c r="J32" s="20"/>
+      <c r="J32" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K32" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L32" s="50" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M32" s="27"/>
       <c r="N32" s="27"/>
       <c r="O32" s="27"/>
-      <c r="P32" s="27"/>
+      <c r="P32" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="33" spans="1:16" ht="110.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="14">
@@ -6192,10 +6626,10 @@
         <v>1712</v>
       </c>
       <c r="D33" s="35" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -6203,19 +6637,23 @@
       <c r="I33" s="20">
         <v>8</v>
       </c>
-      <c r="J33" s="20"/>
+      <c r="J33" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K33" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L33" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M33" s="27"/>
       <c r="N33" s="27"/>
       <c r="O33" s="27"/>
-      <c r="P33" s="27"/>
-    </row>
-    <row r="34" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P33" s="52" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A34" s="14">
         <v>28</v>
       </c>
@@ -6224,7 +6662,7 @@
         <v>1721</v>
       </c>
       <c r="D34" s="35" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E34" s="22"/>
       <c r="F34" s="20"/>
@@ -6233,19 +6671,23 @@
       <c r="I34" s="20">
         <v>1</v>
       </c>
-      <c r="J34" s="20"/>
+      <c r="J34" s="46" t="s">
+        <v>145</v>
+      </c>
       <c r="K34" s="21"/>
       <c r="L34" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M34" s="27">
         <v>1</v>
       </c>
       <c r="N34" s="27"/>
       <c r="O34" s="27"/>
-      <c r="P34" s="27"/>
-    </row>
-    <row r="35" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P34" s="51" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A35" s="14">
         <v>29</v>
       </c>
@@ -6253,7 +6695,7 @@
         <v>2121</v>
       </c>
       <c r="D35" s="35" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E35" s="22"/>
       <c r="F35" s="20"/>
@@ -6262,17 +6704,21 @@
       <c r="I35" s="20">
         <v>1</v>
       </c>
-      <c r="J35" s="20"/>
+      <c r="J35" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K35" s="21"/>
       <c r="L35" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M35" s="27">
         <v>1</v>
       </c>
       <c r="N35" s="27"/>
       <c r="O35" s="27"/>
-      <c r="P35" s="27"/>
+      <c r="P35" s="51" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="36" spans="1:16" ht="137.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="14">
@@ -6282,7 +6728,7 @@
         <v>2111</v>
       </c>
       <c r="D36" s="36" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E36" s="22"/>
       <c r="F36" s="20"/>
@@ -6291,17 +6737,23 @@
       <c r="I36" s="20">
         <v>3</v>
       </c>
-      <c r="J36" s="20"/>
+      <c r="J36" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K36" s="21"/>
-      <c r="L36" s="46" t="s">
-        <v>87</v>
+      <c r="L36" s="56" t="s">
+        <v>139</v>
       </c>
       <c r="M36" s="27"/>
       <c r="N36" s="27"/>
-      <c r="O36" s="27"/>
-      <c r="P36" s="27"/>
-    </row>
-    <row r="37" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="O36" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="P36" s="27" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A37" s="14">
         <v>32</v>
       </c>
@@ -6309,7 +6761,7 @@
         <v>121</v>
       </c>
       <c r="D37" s="35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E37" s="22"/>
       <c r="F37" s="20"/>
@@ -6318,19 +6770,23 @@
       <c r="I37" s="20">
         <v>1</v>
       </c>
-      <c r="J37" s="20"/>
+      <c r="J37" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K37" s="21"/>
       <c r="L37" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M37" s="27">
         <v>1</v>
       </c>
       <c r="N37" s="27"/>
       <c r="O37" s="27"/>
-      <c r="P37" s="27"/>
-    </row>
-    <row r="38" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P37" s="52" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A38" s="14">
         <v>34</v>
       </c>
@@ -6338,7 +6794,7 @@
         <v>122</v>
       </c>
       <c r="D38" s="36" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E38" s="22"/>
       <c r="F38" s="20"/>
@@ -6347,19 +6803,23 @@
       <c r="I38" s="20">
         <v>1</v>
       </c>
-      <c r="J38" s="20"/>
+      <c r="J38" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K38" s="21"/>
       <c r="L38" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M38" s="27">
         <v>1</v>
       </c>
       <c r="N38" s="27"/>
       <c r="O38" s="27"/>
-      <c r="P38" s="27"/>
-    </row>
-    <row r="39" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P38" s="51" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A39" s="14">
         <v>35</v>
       </c>
@@ -6367,7 +6827,7 @@
         <v>123</v>
       </c>
       <c r="D39" s="35" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E39" s="22"/>
       <c r="F39" s="20"/>
@@ -6376,17 +6836,21 @@
       <c r="I39" s="20">
         <v>1</v>
       </c>
-      <c r="J39" s="20"/>
+      <c r="J39" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K39" s="21"/>
       <c r="L39" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M39" s="27">
         <v>1</v>
       </c>
       <c r="N39" s="27"/>
       <c r="O39" s="27"/>
-      <c r="P39" s="27"/>
+      <c r="P39" s="51" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="40" spans="1:16" ht="117" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="14">
@@ -6396,10 +6860,10 @@
         <v>116</v>
       </c>
       <c r="D40" s="35" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F40" s="20"/>
       <c r="G40" s="20"/>
@@ -6407,88 +6871,102 @@
       <c r="I40" s="20">
         <v>6</v>
       </c>
-      <c r="J40" s="20"/>
+      <c r="J40" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K40" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L40" s="45" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M40" s="27"/>
       <c r="N40" s="27"/>
       <c r="O40" s="27"/>
-      <c r="P40" s="27"/>
-    </row>
-    <row r="41" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P40" s="51" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="54" x14ac:dyDescent="0.15">
       <c r="A41" s="14">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C41" s="20">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D41" s="35" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E41" s="22"/>
       <c r="F41" s="20"/>
       <c r="G41" s="20"/>
       <c r="H41" s="22"/>
       <c r="I41" s="20">
-        <v>2</v>
-      </c>
-      <c r="J41" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J41" s="46" t="s">
+        <v>145</v>
+      </c>
       <c r="K41" s="21"/>
       <c r="L41" s="41" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="M41" s="27">
         <v>1</v>
       </c>
       <c r="N41" s="27"/>
       <c r="O41" s="27"/>
-      <c r="P41" s="27"/>
-    </row>
-    <row r="42" spans="1:16" ht="45" x14ac:dyDescent="0.15">
+      <c r="P41" s="51" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="121.5" x14ac:dyDescent="0.15">
       <c r="A42" s="14">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C42" s="20">
-        <v>125</v>
-      </c>
-      <c r="D42" s="35" t="s">
-        <v>62</v>
-      </c>
-      <c r="E42" s="22"/>
+        <v>126</v>
+      </c>
+      <c r="D42" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="E42" s="22" t="s">
+        <v>84</v>
+      </c>
       <c r="F42" s="20"/>
       <c r="G42" s="20"/>
       <c r="H42" s="22"/>
       <c r="I42" s="20">
         <v>1</v>
       </c>
-      <c r="J42" s="20"/>
+      <c r="J42" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K42" s="21"/>
-      <c r="L42" s="41" t="s">
-        <v>79</v>
-      </c>
-      <c r="M42" s="27">
-        <v>1</v>
-      </c>
+      <c r="L42" s="47" t="s">
+        <v>85</v>
+      </c>
+      <c r="M42" s="27"/>
       <c r="N42" s="27"/>
-      <c r="O42" s="27"/>
-      <c r="P42" s="27"/>
-    </row>
-    <row r="43" spans="1:16" ht="121.5" x14ac:dyDescent="0.15">
+      <c r="O42" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="P42" s="27" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="40.5" x14ac:dyDescent="0.15">
       <c r="A43" s="14">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C43" s="20">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D43" s="36" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="F43" s="20"/>
       <c r="G43" s="20"/>
@@ -6496,28 +6974,30 @@
       <c r="I43" s="20">
         <v>1</v>
       </c>
-      <c r="J43" s="20"/>
+      <c r="J43" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K43" s="21"/>
       <c r="L43" s="47" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="M43" s="27"/>
       <c r="N43" s="27"/>
       <c r="O43" s="27"/>
       <c r="P43" s="27"/>
     </row>
-    <row r="44" spans="1:16" ht="40.5" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:16" ht="243" x14ac:dyDescent="0.15">
       <c r="A44" s="14">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C44" s="20">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D44" s="36" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="F44" s="20"/>
       <c r="G44" s="20"/>
@@ -6525,28 +7005,34 @@
       <c r="I44" s="20">
         <v>1</v>
       </c>
-      <c r="J44" s="20"/>
+      <c r="J44" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K44" s="21"/>
       <c r="L44" s="47" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="M44" s="27"/>
       <c r="N44" s="27"/>
-      <c r="O44" s="27"/>
-      <c r="P44" s="27"/>
-    </row>
-    <row r="45" spans="1:16" ht="243" x14ac:dyDescent="0.15">
+      <c r="O44" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="P44" s="27" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="162" x14ac:dyDescent="0.15">
       <c r="A45" s="14">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C45" s="20">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D45" s="36" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F45" s="20"/>
       <c r="G45" s="20"/>
@@ -6554,166 +7040,198 @@
       <c r="I45" s="20">
         <v>1</v>
       </c>
-      <c r="J45" s="20"/>
+      <c r="J45" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K45" s="21"/>
       <c r="L45" s="47" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="M45" s="27"/>
       <c r="N45" s="27"/>
-      <c r="O45" s="27"/>
-      <c r="P45" s="27"/>
+      <c r="O45" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="P45" s="27" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="46" spans="1:16" ht="162" x14ac:dyDescent="0.15">
       <c r="A46" s="14">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C46" s="20">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D46" s="36" t="s">
-        <v>99</v>
-      </c>
-      <c r="E46" s="22" t="s">
-        <v>100</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="E46" s="22"/>
       <c r="F46" s="20"/>
       <c r="G46" s="20"/>
       <c r="H46" s="22"/>
       <c r="I46" s="20">
         <v>1</v>
       </c>
-      <c r="J46" s="20"/>
+      <c r="J46" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K46" s="21"/>
       <c r="L46" s="47" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="M46" s="27"/>
       <c r="N46" s="27"/>
-      <c r="O46" s="27"/>
-      <c r="P46" s="27"/>
-    </row>
-    <row r="47" spans="1:16" ht="162" x14ac:dyDescent="0.15">
+      <c r="O46" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="P46" s="27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="256.5" x14ac:dyDescent="0.15">
       <c r="A47" s="14">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C47" s="20">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D47" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="E47" s="22"/>
+        <v>106</v>
+      </c>
+      <c r="E47" s="22" t="s">
+        <v>107</v>
+      </c>
       <c r="F47" s="20"/>
       <c r="G47" s="20"/>
       <c r="H47" s="22"/>
       <c r="I47" s="20">
-        <v>1</v>
-      </c>
-      <c r="J47" s="20"/>
+        <v>50</v>
+      </c>
+      <c r="J47" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K47" s="21"/>
       <c r="L47" s="47" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="M47" s="27"/>
       <c r="N47" s="27"/>
-      <c r="O47" s="27"/>
-      <c r="P47" s="27"/>
-    </row>
-    <row r="48" spans="1:16" ht="256.5" x14ac:dyDescent="0.15">
+      <c r="O47" s="27" t="s">
+        <v>114</v>
+      </c>
+      <c r="P47" s="27" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="243" x14ac:dyDescent="0.15">
       <c r="A48" s="14">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C48" s="20">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D48" s="36" t="s">
-        <v>114</v>
-      </c>
-      <c r="E48" s="22" t="s">
-        <v>115</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="E48" s="22"/>
       <c r="F48" s="20"/>
       <c r="G48" s="20"/>
       <c r="H48" s="22"/>
       <c r="I48" s="20">
-        <v>50</v>
-      </c>
-      <c r="J48" s="20"/>
+        <v>1</v>
+      </c>
+      <c r="J48" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K48" s="21"/>
       <c r="L48" s="47" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="M48" s="27"/>
       <c r="N48" s="27"/>
-      <c r="O48" s="27"/>
-      <c r="P48" s="27"/>
-    </row>
-    <row r="49" spans="1:16" ht="243" x14ac:dyDescent="0.15">
+      <c r="O48" s="27" t="s">
+        <v>113</v>
+      </c>
+      <c r="P48" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="15" x14ac:dyDescent="0.15">
       <c r="A49" s="14">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C49" s="20">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D49" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="E49" s="22"/>
+        <v>99</v>
+      </c>
+      <c r="E49" s="22" t="s">
+        <v>101</v>
+      </c>
       <c r="F49" s="20"/>
       <c r="G49" s="20"/>
       <c r="H49" s="22"/>
       <c r="I49" s="20">
         <v>1</v>
       </c>
-      <c r="J49" s="20"/>
+      <c r="J49" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K49" s="21"/>
-      <c r="L49" s="47" t="s">
-        <v>105</v>
+      <c r="L49" s="41" t="s">
+        <v>100</v>
       </c>
       <c r="M49" s="27"/>
       <c r="N49" s="27"/>
       <c r="O49" s="27"/>
-      <c r="P49" s="27"/>
+      <c r="P49" s="51" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="50" spans="1:16" ht="15" x14ac:dyDescent="0.15">
       <c r="A50" s="14">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C50" s="20">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D50" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="E50" s="22" t="s">
-        <v>109</v>
-      </c>
+        <v>102</v>
+      </c>
+      <c r="E50" s="22"/>
       <c r="F50" s="20"/>
       <c r="G50" s="20"/>
       <c r="H50" s="22"/>
       <c r="I50" s="20">
         <v>1</v>
       </c>
-      <c r="J50" s="20"/>
-      <c r="K50" s="21"/>
+      <c r="J50" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="K50" s="49" t="s">
+        <v>111</v>
+      </c>
       <c r="L50" s="41" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="M50" s="27"/>
       <c r="N50" s="27"/>
       <c r="O50" s="27"/>
-      <c r="P50" s="27"/>
+      <c r="P50" s="51" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="51" spans="1:16" ht="15" x14ac:dyDescent="0.15">
       <c r="A51" s="14">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C51" s="20">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D51" s="36" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E51" s="22"/>
       <c r="F51" s="20"/>
@@ -6722,27 +7240,31 @@
       <c r="I51" s="20">
         <v>1</v>
       </c>
-      <c r="J51" s="20"/>
+      <c r="J51" s="46" t="s">
+        <v>145</v>
+      </c>
       <c r="K51" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L51" s="41" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M51" s="27"/>
       <c r="N51" s="27"/>
       <c r="O51" s="27"/>
-      <c r="P51" s="27"/>
+      <c r="P51" s="51" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="52" spans="1:16" ht="15" x14ac:dyDescent="0.15">
       <c r="A52" s="14">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C52" s="20">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D52" s="36" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E52" s="22"/>
       <c r="F52" s="20"/>
@@ -6751,83 +7273,102 @@
       <c r="I52" s="20">
         <v>1</v>
       </c>
-      <c r="J52" s="20"/>
+      <c r="J52" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K52" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L52" s="41" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M52" s="27"/>
       <c r="N52" s="27"/>
       <c r="O52" s="27"/>
-      <c r="P52" s="27"/>
+      <c r="P52" s="52" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="53" spans="1:16" ht="15" x14ac:dyDescent="0.15">
       <c r="A53" s="14">
         <v>50</v>
       </c>
       <c r="C53" s="20">
-        <v>136</v>
+        <v>1312</v>
       </c>
       <c r="D53" s="36" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="E53" s="22"/>
       <c r="F53" s="20"/>
       <c r="G53" s="20"/>
       <c r="H53" s="22"/>
       <c r="I53" s="20">
-        <v>1</v>
-      </c>
-      <c r="J53" s="20"/>
+        <v>2</v>
+      </c>
+      <c r="J53" s="55" t="s">
+        <v>146</v>
+      </c>
       <c r="K53" s="49" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="L53" s="41" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="M53" s="27"/>
       <c r="N53" s="27"/>
       <c r="O53" s="27"/>
-      <c r="P53" s="27"/>
-    </row>
-    <row r="54" spans="1:16" ht="15" x14ac:dyDescent="0.15">
+      <c r="P53" s="51" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" ht="58.5" x14ac:dyDescent="0.15">
       <c r="A54" s="14">
         <v>50</v>
       </c>
       <c r="C54" s="20">
-        <v>1312</v>
+        <v>3129</v>
       </c>
       <c r="D54" s="36" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E54" s="22"/>
       <c r="F54" s="20"/>
       <c r="G54" s="20"/>
       <c r="H54" s="22"/>
       <c r="I54" s="20">
-        <v>2</v>
-      </c>
-      <c r="J54" s="20"/>
-      <c r="K54" s="49" t="s">
-        <v>119</v>
-      </c>
-      <c r="L54" s="41" t="s">
-        <v>111</v>
+        <v>1</v>
+      </c>
+      <c r="J54" s="55" t="s">
+        <v>146</v>
+      </c>
+      <c r="K54" s="49"/>
+      <c r="L54" s="42" t="s">
+        <v>73</v>
       </c>
       <c r="M54" s="27"/>
       <c r="N54" s="27"/>
       <c r="O54" s="27"/>
-      <c r="P54" s="27"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="P54" s="51" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" ht="28.5" x14ac:dyDescent="0.15">
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.15">
+      <c r="O55" s="53" t="s">
+        <v>124</v>
+      </c>
+      <c r="P55" s="10" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="28.5" x14ac:dyDescent="0.15">
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
+      <c r="O56" s="53" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.15">
       <c r="I57" s="2"/>
@@ -11485,26 +12026,15 @@
       <c r="I1220" s="2"/>
       <c r="J1220" s="2"/>
     </row>
-    <row r="1221" spans="9:10" x14ac:dyDescent="0.15">
-      <c r="I1221" s="2"/>
-      <c r="J1221" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="N1:P1"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="C3:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:H1"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
     <mergeCell ref="O5:O6"/>
@@ -11521,23 +12051,31 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="L4:M4"/>
     <mergeCell ref="N4:P4"/>
-    <mergeCell ref="A1:A4"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="C3:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="L1:M1"/>
   </mergeCells>
   <phoneticPr fontId="61" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="L43" r:id="rId1" xr:uid="{9A51B0C7-8481-4F5F-96C9-71A2DF3DDCA7}"/>
-    <hyperlink ref="L44" r:id="rId2" xr:uid="{BC501510-C86E-4A45-BAA8-5F5E22C20442}"/>
-    <hyperlink ref="L45" r:id="rId3" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1563820041%3AH%3AjEXVXFz29uWhSPA32SdLxq18tbGVRP6N%3Ab1e44a53e68312397166bdb38376f31f&amp;ali_trackid=318_b1e44a53e68312397166bdb38376f31f&amp;id=668804973431&amp;mi_id=0000kh4JsEhs_IKQwaZwLe5GPzZBrKEtnqIAl4nMzgEcpGs&amp;mm_sceneid=0_0_2198670068_0&amp;priceTId=213e097817677727727551092e11ab&amp;skuId=6072168990782&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%220ce0092ebee4bb5c990e1ed0aae83472%22%7D&amp;xxc=ad_ztc" xr:uid="{EE7187D2-5C29-4C71-8BF0-14CC690401EB}"/>
-    <hyperlink ref="L46" r:id="rId4" display="https://item.taobao.com/item.htm?abbucket=15&amp;id=684180101591&amp;mi_id=0000kHsnKO9vrl_xXRKAYuWwfk1ZxpJzkY1oGgmAntBdN2A&amp;ns=1&amp;priceTId=215040db17693197452846906e10bd&amp;skuId=5066190559427&amp;spm=a21n57.1.hoverItem.13&amp;utparam=%7B%22aplus_abtest%22%3A%2200fb48171d68baf920a6c2997ba800f5%22%7D&amp;xxc=taobaoSearch" xr:uid="{640829AA-10E2-4344-B84B-AF14836FC0FA}"/>
-    <hyperlink ref="L47" r:id="rId5" display="https://item.taobao.com/item.htm?abbucket=15&amp;id=885444239746&amp;mi_id=00004gN7JSgLTLqH9NscZa5BV-fDjGIRhn7dS2llqgBEm-I&amp;ns=1&amp;priceTId=215040db17693199893824488e10bd&amp;skuId=5729109569961&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%220d184a79d8dee207c56cd615483888e0%22%7D&amp;xxc=taobaoSearch" xr:uid="{D9E14E51-6908-4600-BF1B-1BE5E52130FA}"/>
-    <hyperlink ref="L49" r:id="rId6" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1202830031%3AH%3A5NEVSZWkfH5vk10Gx8WsEg%3D%3D%3A0e3224a199436b146fadd1013df40d50&amp;ali_trackid=282_0e3224a199436b146fadd1013df40d50&amp;id=589213401941&amp;mi_id=0000tXboOyQ6vKwx8WiuBo_0I904yCwGgBZQ-DEtp9Eidvc&amp;mm_sceneid=1_0_343370108_0&amp;priceTId=214782f517694062736734983e1fe1&amp;skuId=4715656587781&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%2243f96ce6df79319aabdbd4973057b1b5%22%7D&amp;xxc=ad_ztc" xr:uid="{A4FE5950-5A28-4F3D-B42C-E6D6ECC79B08}"/>
-    <hyperlink ref="L48" r:id="rId7" display="https://item.taobao.com/item.htm?ali_refid=a3_430673_1006%3A1109974134%3AH%3AS9mt8%2FS9IPRAnlGXK23dCRerfi2%2BAYZj%3A75421c7a1bf937df626379b8de81db84&amp;ali_trackid=282_75421c7a1bf937df626379b8de81db84&amp;id=774427618182&amp;loginBonus=1&amp;mi_id=0000OtzXamOT9vAra9TbUQiBvRLBsdZJRcmzsekmz3yUyS0&amp;mm_sceneid=1_0_99588015_0&amp;priceTId=2150467817696032421462002e22b0&amp;skuId=5300832301565&amp;spm=a21n57.sem.item.4&amp;utparam=%7B%22aplus_abtest%22%3A%22c7bbb9e8de08729fc098be83e797fb13%22%7D&amp;xxc=ad_ztc" xr:uid="{FC3750A0-F3B8-4313-B9DE-37439F3E109E}"/>
+    <hyperlink ref="L42" r:id="rId1" xr:uid="{9A51B0C7-8481-4F5F-96C9-71A2DF3DDCA7}"/>
+    <hyperlink ref="L43" r:id="rId2" xr:uid="{BC501510-C86E-4A45-BAA8-5F5E22C20442}"/>
+    <hyperlink ref="L44" r:id="rId3" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1563820041%3AH%3AjEXVXFz29uWhSPA32SdLxq18tbGVRP6N%3Ab1e44a53e68312397166bdb38376f31f&amp;ali_trackid=318_b1e44a53e68312397166bdb38376f31f&amp;id=668804973431&amp;mi_id=0000kh4JsEhs_IKQwaZwLe5GPzZBrKEtnqIAl4nMzgEcpGs&amp;mm_sceneid=0_0_2198670068_0&amp;priceTId=213e097817677727727551092e11ab&amp;skuId=6072168990782&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%220ce0092ebee4bb5c990e1ed0aae83472%22%7D&amp;xxc=ad_ztc" xr:uid="{EE7187D2-5C29-4C71-8BF0-14CC690401EB}"/>
+    <hyperlink ref="L45" r:id="rId4" display="https://item.taobao.com/item.htm?abbucket=15&amp;id=684180101591&amp;mi_id=0000kHsnKO9vrl_xXRKAYuWwfk1ZxpJzkY1oGgmAntBdN2A&amp;ns=1&amp;priceTId=215040db17693197452846906e10bd&amp;skuId=5066190559427&amp;spm=a21n57.1.hoverItem.13&amp;utparam=%7B%22aplus_abtest%22%3A%2200fb48171d68baf920a6c2997ba800f5%22%7D&amp;xxc=taobaoSearch" xr:uid="{640829AA-10E2-4344-B84B-AF14836FC0FA}"/>
+    <hyperlink ref="L46" r:id="rId5" display="https://item.taobao.com/item.htm?abbucket=15&amp;id=885444239746&amp;mi_id=00004gN7JSgLTLqH9NscZa5BV-fDjGIRhn7dS2llqgBEm-I&amp;ns=1&amp;priceTId=215040db17693199893824488e10bd&amp;skuId=5729109569961&amp;spm=a21n57.1.hoverItem.3&amp;utparam=%7B%22aplus_abtest%22%3A%220d184a79d8dee207c56cd615483888e0%22%7D&amp;xxc=taobaoSearch" xr:uid="{D9E14E51-6908-4600-BF1B-1BE5E52130FA}"/>
+    <hyperlink ref="L48" r:id="rId6" display="https://detail.tmall.com/item.htm?ali_refid=a3_430582_1006%3A1202830031%3AH%3A5NEVSZWkfH5vk10Gx8WsEg%3D%3D%3A0e3224a199436b146fadd1013df40d50&amp;ali_trackid=282_0e3224a199436b146fadd1013df40d50&amp;id=589213401941&amp;mi_id=0000tXboOyQ6vKwx8WiuBo_0I904yCwGgBZQ-DEtp9Eidvc&amp;mm_sceneid=1_0_343370108_0&amp;priceTId=214782f517694062736734983e1fe1&amp;skuId=4715656587781&amp;spm=a21n57.1.hoverItem.1&amp;utparam=%7B%22aplus_abtest%22%3A%2243f96ce6df79319aabdbd4973057b1b5%22%7D&amp;xxc=ad_ztc" xr:uid="{A4FE5950-5A28-4F3D-B42C-E6D6ECC79B08}"/>
+    <hyperlink ref="L47" r:id="rId7" display="https://item.taobao.com/item.htm?ali_refid=a3_430673_1006%3A1109974134%3AH%3AS9mt8%2FS9IPRAnlGXK23dCRerfi2%2BAYZj%3A75421c7a1bf937df626379b8de81db84&amp;ali_trackid=282_75421c7a1bf937df626379b8de81db84&amp;id=774427618182&amp;loginBonus=1&amp;mi_id=0000OtzXamOT9vAra9TbUQiBvRLBsdZJRcmzsekmz3yUyS0&amp;mm_sceneid=1_0_99588015_0&amp;priceTId=2150467817696032421462002e22b0&amp;skuId=5300832301565&amp;spm=a21n57.sem.item.4&amp;utparam=%7B%22aplus_abtest%22%3A%22c7bbb9e8de08729fc098be83e797fb13%22%7D&amp;xxc=ad_ztc" xr:uid="{FC3750A0-F3B8-4313-B9DE-37439F3E109E}"/>
+    <hyperlink ref="L36" r:id="rId8" xr:uid="{B9066E40-3620-40FD-976E-186331CB00E7}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>

</xml_diff>